<commit_message>
Add sales delete flow and local Excel fallback
</commit_message>
<xml_diff>
--- a/data/sales.xlsx
+++ b/data/sales.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="66">
   <si>
     <t>ITEM NAME</t>
   </si>
@@ -188,53 +188,41 @@
     <t>SALE VALUE</t>
   </si>
   <si>
-    <t>2026-08-28</t>
+    <t>OPENING VALUE</t>
+  </si>
+  <si>
+    <t>SUPPLY</t>
+  </si>
+  <si>
+    <t>SUPPLY VALUE</t>
+  </si>
+  <si>
+    <t>TOTAL STOCK</t>
+  </si>
+  <si>
+    <t>TOTAL VALUE</t>
+  </si>
+  <si>
+    <t>SALES QUANTITY</t>
+  </si>
+  <si>
+    <t>CLOSING STOCK</t>
+  </si>
+  <si>
+    <t>CLOSING VALUE</t>
   </si>
   <si>
     <t>2026-08</t>
   </si>
   <si>
-    <t>OPENING VALUE</t>
-  </si>
-  <si>
-    <t>SUPPLY</t>
-  </si>
-  <si>
-    <t>SUPPLY VALUE</t>
-  </si>
-  <si>
-    <t>TOTAL STOCK</t>
-  </si>
-  <si>
-    <t>TOTAL VALUE</t>
-  </si>
-  <si>
-    <t>SALES QUANTITY</t>
-  </si>
-  <si>
-    <t>CLOSING STOCK</t>
-  </si>
-  <si>
-    <t>CLOSING VALUE</t>
-  </si>
-  <si>
     <t>Shikaki Hairwash - 200 ML</t>
-  </si>
-  <si>
-    <t>SALES - 28 AUGUST 2026</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>DAILY TOTAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -244,10 +232,6 @@
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -297,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -305,7 +289,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1216,7 +1199,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1249,106 +1232,6 @@
     <row r="2" spans="1:6" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5">
-        <v>95</v>
-      </c>
-      <c r="E5">
-        <v>3</v>
-      </c>
-      <c r="F5">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>48</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7">
-        <v>22</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8">
-        <v>200</v>
-      </c>
-      <c r="E8">
-        <v>15</v>
-      </c>
-      <c r="F8">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9">
-        <v>1563</v>
-      </c>
-      <c r="E9">
-        <v>4</v>
-      </c>
-      <c r="F9">
-        <v>6252</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -1387,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1396,132 +1279,7 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4">
-        <v>95</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5">
-        <v>48</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6">
-        <v>22</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7">
-        <v>200</v>
-      </c>
-      <c r="D7">
-        <v>15</v>
-      </c>
-      <c r="E7">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>1563</v>
-      </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-      <c r="E8">
-        <v>6252</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D9" s="4">
-        <v>24</v>
-      </c>
-      <c r="E9" s="4">
-        <v>9607</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1559,36 +1317,36 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>63</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1615,21 +1373,21 @@
         <v>6252</v>
       </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
         <v>4</v>
       </c>
-      <c r="K2">
+      <c r="M2">
         <v>6252</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -1670,7 +1428,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -1711,7 +1469,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -1752,7 +1510,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1793,7 +1551,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -1834,7 +1592,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -1861,21 +1619,21 @@
         <v>1386</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M8">
-        <v>1364</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -1916,7 +1674,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
@@ -1943,21 +1701,21 @@
         <v>4896</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M10">
-        <v>4848</v>
+        <v>4896</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
@@ -1998,7 +1756,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
@@ -2039,7 +1797,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -2080,7 +1838,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
@@ -2121,7 +1879,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -2162,7 +1920,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
@@ -2203,7 +1961,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
@@ -2244,7 +2002,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
@@ -2285,7 +2043,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
@@ -2326,7 +2084,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B20" t="s">
         <v>21</v>
@@ -2367,7 +2125,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
         <v>22</v>
@@ -2408,7 +2166,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
         <v>23</v>
@@ -2449,7 +2207,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
         <v>24</v>
@@ -2490,7 +2248,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
         <v>25</v>
@@ -2531,7 +2289,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
         <v>26</v>
@@ -2572,7 +2330,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s">
         <v>27</v>
@@ -2613,7 +2371,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
@@ -2654,7 +2412,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B28" t="s">
         <v>29</v>
@@ -2695,7 +2453,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
         <v>30</v>
@@ -2736,7 +2494,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
         <v>31</v>
@@ -2777,7 +2535,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
@@ -2818,7 +2576,7 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
@@ -2845,21 +2603,21 @@
         <v>2280</v>
       </c>
       <c r="J32">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K32">
-        <v>285</v>
+        <v>0</v>
       </c>
       <c r="L32">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="M32">
-        <v>1995</v>
+        <v>2280</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
@@ -2900,7 +2658,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
         <v>35</v>
@@ -2941,10 +2699,10 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C35">
         <v>105</v>
@@ -2982,7 +2740,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B36" t="s">
         <v>37</v>
@@ -3023,7 +2781,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B37" t="s">
         <v>38</v>
@@ -3064,7 +2822,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B38" t="s">
         <v>39</v>
@@ -3105,7 +2863,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B39" t="s">
         <v>40</v>
@@ -3132,21 +2890,21 @@
         <v>30200</v>
       </c>
       <c r="J39">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K39">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="L39">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="M39">
-        <v>27200</v>
+        <v>30200</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B40" t="s">
         <v>41</v>
@@ -3187,7 +2945,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B41" t="s">
         <v>42</v>
@@ -3228,7 +2986,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B42" t="s">
         <v>43</v>
@@ -3269,7 +3027,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B43" t="s">
         <v>44</v>
@@ -3310,7 +3068,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B44" t="s">
         <v>45</v>
@@ -3351,7 +3109,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B45" t="s">
         <v>46</v>
@@ -3392,7 +3150,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B46" t="s">
         <v>47</v>
@@ -3433,7 +3191,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B47" t="s">
         <v>48</v>
@@ -3474,7 +3232,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B48" t="s">
         <v>49</v>
@@ -3515,7 +3273,7 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B49" t="s">
         <v>50</v>
@@ -3556,7 +3314,7 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B50" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
changes happend on deletion thing
</commit_message>
<xml_diff>
--- a/data/sales.xlsx
+++ b/data/sales.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="70">
   <si>
     <t>ITEM NAME</t>
   </si>
@@ -188,6 +188,12 @@
     <t>SALE VALUE</t>
   </si>
   <si>
+    <t>2026-08-25</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
     <t>OPENING VALUE</t>
   </si>
   <si>
@@ -212,17 +218,23 @@
     <t>CLOSING VALUE</t>
   </si>
   <si>
-    <t>2026-08</t>
-  </si>
-  <si>
     <t>Shikaki Hairwash - 200 ML</t>
+  </si>
+  <si>
+    <t>SALES - 25 AUGUST 2026</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>DAILY TOTAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -232,6 +244,10 @@
     </font>
     <font>
       <b/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="4">
@@ -281,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -289,6 +305,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1199,7 +1216,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1232,6 +1249,26 @@
     <row r="2" spans="1:6" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>180</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>180</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -1270,7 +1307,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1279,7 +1316,64 @@
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4">
+        <v>180</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1317,36 +1411,36 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -1387,7 +1481,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -1428,7 +1522,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
@@ -1455,21 +1549,21 @@
         <v>19260</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="L4">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M4">
-        <v>19260</v>
+        <v>19080</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -1510,7 +1604,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1551,7 +1645,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
@@ -1592,7 +1686,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -1633,7 +1727,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
@@ -1674,7 +1768,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
         <v>11</v>
@@ -1715,7 +1809,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
@@ -1756,7 +1850,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
@@ -1797,7 +1891,7 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
@@ -1838,7 +1932,7 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
         <v>15</v>
@@ -1879,7 +1973,7 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -1920,7 +2014,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
@@ -1961,7 +2055,7 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
         <v>18</v>
@@ -2002,7 +2096,7 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
         <v>19</v>
@@ -2043,7 +2137,7 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
@@ -2084,7 +2178,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B20" t="s">
         <v>21</v>
@@ -2125,7 +2219,7 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
         <v>22</v>
@@ -2166,7 +2260,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B22" t="s">
         <v>23</v>
@@ -2207,7 +2301,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B23" t="s">
         <v>24</v>
@@ -2248,7 +2342,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
         <v>25</v>
@@ -2289,7 +2383,7 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
         <v>26</v>
@@ -2330,7 +2424,7 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
         <v>27</v>
@@ -2371,7 +2465,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
@@ -2412,7 +2506,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B28" t="s">
         <v>29</v>
@@ -2453,7 +2547,7 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
         <v>30</v>
@@ -2494,7 +2588,7 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B30" t="s">
         <v>31</v>
@@ -2535,7 +2629,7 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B31" t="s">
         <v>32</v>
@@ -2576,7 +2670,7 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
@@ -2617,7 +2711,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B33" t="s">
         <v>34</v>
@@ -2658,7 +2752,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
         <v>35</v>
@@ -2699,10 +2793,10 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C35">
         <v>105</v>
@@ -2740,7 +2834,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B36" t="s">
         <v>37</v>
@@ -2781,7 +2875,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
         <v>38</v>
@@ -2822,7 +2916,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
         <v>39</v>
@@ -2863,7 +2957,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B39" t="s">
         <v>40</v>
@@ -2904,7 +2998,7 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
         <v>41</v>
@@ -2945,7 +3039,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
         <v>42</v>
@@ -2986,7 +3080,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B42" t="s">
         <v>43</v>
@@ -3027,7 +3121,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
         <v>44</v>
@@ -3068,7 +3162,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
         <v>45</v>
@@ -3109,7 +3203,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B45" t="s">
         <v>46</v>
@@ -3150,7 +3244,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B46" t="s">
         <v>47</v>
@@ -3191,7 +3285,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B47" t="s">
         <v>48</v>
@@ -3232,7 +3326,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B48" t="s">
         <v>49</v>
@@ -3273,7 +3367,7 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B49" t="s">
         <v>50</v>
@@ -3314,7 +3408,7 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B50" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Fix: Daily sales report date filtering and button sizing
- Fixed date format matching in daily sales report filter
- Updated CSS for consistent button heights (43px)
- Both Generate Report and Download PDF buttons now same size
</commit_message>
<xml_diff>
--- a/data/sales.xlsx
+++ b/data/sales.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="72">
   <si>
     <t>ITEM NAME</t>
   </si>
@@ -194,6 +194,9 @@
     <t>2026-08</t>
   </si>
   <si>
+    <t>2026-08-30</t>
+  </si>
+  <si>
     <t>OPENING VALUE</t>
   </si>
   <si>
@@ -228,6 +231,9 @@
   </si>
   <si>
     <t>DAILY TOTAL</t>
+  </si>
+  <si>
+    <t>SALES - 30 AUGUST 2026</t>
   </si>
 </sst>
 </file>
@@ -1216,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1267,6 +1273,46 @@
       </c>
       <c r="F5">
         <v>180</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>1563</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>1563</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>3126</v>
       </c>
     </row>
   </sheetData>
@@ -1307,7 +1353,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1319,7 +1365,7 @@
   <sheetData>
     <row r="1" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1356,21 +1402,94 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="4" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>1563</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D5" s="4">
+      <c r="B6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1743</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="4">
-        <v>180</v>
+      <c r="D11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>1563</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12">
+        <v>3126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2</v>
+      </c>
+      <c r="E13" s="4">
+        <v>3126</v>
       </c>
     </row>
   </sheetData>
@@ -1411,31 +1530,31 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>55</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1467,16 +1586,16 @@
         <v>6252</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>4689</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>6252</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2796,7 +2915,7 @@
         <v>57</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C35">
         <v>105</v>

</xml_diff>